<commit_message>
[CI] [79466]  <wifi> <feat> support system persist config - PM
</commit_message>
<xml_diff>
--- a/middleware/soc/bk7239n/sys_persist_config.xlsx
+++ b/middleware/soc/bk7239n/sys_persist_config.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="212">
   <si>
     <t xml:space="preserve">space</t>
   </si>
@@ -612,10 +612,97 @@
     <t xml:space="preserve">pm</t>
   </si>
   <si>
-    <t xml:space="preserve">vdddig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vddana</t>
+    <t xml:space="preserve">wifipll_vanaldosel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0xF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wifipll_hpssren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wifipll_anabufsel_tx1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wifipll_anabufsel_tx0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wifipll_anabufsel_rx1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wifipll_anabufsel_rx0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">btpll_vanaldosel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">btpll_hpssren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">btpll_anabufsel_tx1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">btpll_anabufsel_tx0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">btpll_anabufsel_rx1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">btpll_anabufsel_rx0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_vanaldosel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_dldohp_high_temp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_aldohp_high_temp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_dldohp_low_temp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_aldohp_low_temp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_bypassen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_ioldolp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_iburstsel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_mrosci_cal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_avea_sel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lvsleep_vcorehsel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0x6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vcorelsel</t>
   </si>
   <si>
     <t xml:space="preserve">tlv_base</t>
@@ -646,9 +733,6 @@
   </si>
   <si>
     <t xml:space="preserve">0xFF000000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0x3</t>
   </si>
   <si>
     <t xml:space="preserve">0x0000FF00</t>
@@ -901,7 +985,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="6.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="6.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="12.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="12.57"/>
@@ -3295,8 +3379,8 @@
       <c r="D119" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="E119" s="6" t="n">
-        <v>1</v>
+      <c r="E119" s="6" t="s">
+        <v>168</v>
       </c>
       <c r="F119" s="5"/>
       <c r="G119" s="5"/>
@@ -3313,10 +3397,10 @@
         <v>1</v>
       </c>
       <c r="D120" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="E120" s="6" t="n">
-        <v>2</v>
+        <v>169</v>
+      </c>
+      <c r="E120" s="6" t="s">
+        <v>170</v>
       </c>
       <c r="F120" s="5"/>
       <c r="G120" s="5"/>
@@ -3330,13 +3414,13 @@
         <v>554</v>
       </c>
       <c r="C121" s="6" t="n">
-        <v>118</v>
+        <v>1</v>
       </c>
       <c r="D121" s="5" t="s">
-        <v>21</v>
+        <v>171</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>22</v>
+        <v>170</v>
       </c>
       <c r="F121" s="5"/>
       <c r="G121" s="5"/>
@@ -3344,18 +3428,15 @@
       <c r="I121" s="5"/>
     </row>
     <row r="122" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A122" s="5" t="s">
-        <v>169</v>
-      </c>
+      <c r="A122" s="5"/>
       <c r="B122" s="6" t="n">
-        <f aca="false">B121+C121</f>
-        <v>672</v>
+        <v>555</v>
       </c>
       <c r="C122" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>24</v>
+        <v>172</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>170</v>
@@ -3368,17 +3449,16 @@
     <row r="123" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="5"/>
       <c r="B123" s="6" t="n">
-        <f aca="false">B122+C122</f>
-        <v>680</v>
+        <v>556</v>
       </c>
       <c r="C123" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D123" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F123" s="5"/>
       <c r="G123" s="5"/>
@@ -3388,17 +3468,16 @@
     <row r="124" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="5"/>
       <c r="B124" s="6" t="n">
-        <f aca="false">B123+C123</f>
-        <v>682</v>
+        <v>557</v>
       </c>
       <c r="C124" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D124" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E124" s="6" t="n">
-        <v>4</v>
+        <v>174</v>
+      </c>
+      <c r="E124" s="6" t="s">
+        <v>170</v>
       </c>
       <c r="F124" s="5"/>
       <c r="G124" s="5"/>
@@ -3408,17 +3487,16 @@
     <row r="125" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="5"/>
       <c r="B125" s="6" t="n">
-        <f aca="false">B124+C124</f>
-        <v>684</v>
+        <v>558</v>
       </c>
       <c r="C125" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E125" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F125" s="5"/>
       <c r="G125" s="5"/>
@@ -3428,17 +3506,16 @@
     <row r="126" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="5"/>
       <c r="B126" s="6" t="n">
-        <f aca="false">B125+C125</f>
-        <v>688</v>
+        <v>559</v>
       </c>
       <c r="C126" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F126" s="5"/>
       <c r="G126" s="5"/>
@@ -3448,17 +3525,16 @@
     <row r="127" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="5"/>
       <c r="B127" s="6" t="n">
-        <f aca="false">B126+C126</f>
-        <v>690</v>
+        <v>560</v>
       </c>
       <c r="C127" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E127" s="6" t="n">
-        <v>24</v>
+        <v>179</v>
+      </c>
+      <c r="E127" s="6" t="s">
+        <v>178</v>
       </c>
       <c r="F127" s="5"/>
       <c r="G127" s="5"/>
@@ -3468,65 +3544,54 @@
     <row r="128" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="5"/>
       <c r="B128" s="6" t="n">
-        <f aca="false">B127+C127</f>
-        <v>692</v>
+        <v>561</v>
       </c>
       <c r="C128" s="6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E128" s="6"/>
-      <c r="F128" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="G128" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="H128" s="6" t="s">
-        <v>179</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="E128" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F128" s="5"/>
+      <c r="G128" s="5"/>
+      <c r="H128" s="6"/>
       <c r="I128" s="5"/>
     </row>
     <row r="129" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="5"/>
       <c r="B129" s="6" t="n">
-        <f aca="false">B128+C128</f>
-        <v>704</v>
+        <v>562</v>
       </c>
       <c r="C129" s="6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E129" s="6"/>
-      <c r="F129" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="G129" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H129" s="6" t="s">
         <v>181</v>
       </c>
+      <c r="E129" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F129" s="5"/>
+      <c r="G129" s="5"/>
+      <c r="H129" s="6"/>
       <c r="I129" s="5"/>
     </row>
     <row r="130" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="5"/>
       <c r="B130" s="6" t="n">
-        <f aca="false">B129+C129</f>
-        <v>716</v>
+        <v>563</v>
       </c>
       <c r="C130" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D130" s="5" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="F130" s="5"/>
       <c r="G130" s="5"/>
@@ -3536,17 +3601,16 @@
     <row r="131" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="5"/>
       <c r="B131" s="6" t="n">
-        <f aca="false">B130+C130</f>
-        <v>718</v>
+        <v>564</v>
       </c>
       <c r="C131" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D131" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E131" s="6" t="n">
-        <v>24</v>
+        <v>183</v>
+      </c>
+      <c r="E131" s="6" t="s">
+        <v>184</v>
       </c>
       <c r="F131" s="5"/>
       <c r="G131" s="5"/>
@@ -3556,53 +3620,512 @@
     <row r="132" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="5"/>
       <c r="B132" s="6" t="n">
-        <f aca="false">B131+C131</f>
-        <v>720</v>
+        <v>565</v>
       </c>
       <c r="C132" s="6" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F132" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="G132" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="H132" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="F132" s="5"/>
+      <c r="G132" s="5"/>
+      <c r="H132" s="6"/>
       <c r="I132" s="5"/>
     </row>
-    <row r="133" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="5"/>
       <c r="B133" s="6" t="n">
-        <f aca="false">B132+C132</f>
+        <v>566</v>
+      </c>
+      <c r="C133" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E133" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F133" s="5"/>
+      <c r="G133" s="5"/>
+      <c r="H133" s="6"/>
+      <c r="I133" s="5"/>
+    </row>
+    <row r="134" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A134" s="5"/>
+      <c r="B134" s="6" t="n">
+        <v>567</v>
+      </c>
+      <c r="C134" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E134" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F134" s="5"/>
+      <c r="G134" s="5"/>
+      <c r="H134" s="6"/>
+      <c r="I134" s="5"/>
+    </row>
+    <row r="135" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A135" s="5"/>
+      <c r="B135" s="6" t="n">
+        <v>568</v>
+      </c>
+      <c r="C135" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="E135" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F135" s="5"/>
+      <c r="G135" s="5"/>
+      <c r="H135" s="6"/>
+      <c r="I135" s="5"/>
+    </row>
+    <row r="136" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A136" s="5"/>
+      <c r="B136" s="6" t="n">
+        <v>569</v>
+      </c>
+      <c r="C136" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="E136" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F136" s="5"/>
+      <c r="G136" s="5"/>
+      <c r="H136" s="6"/>
+      <c r="I136" s="5"/>
+    </row>
+    <row r="137" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A137" s="5"/>
+      <c r="B137" s="6" t="n">
+        <v>570</v>
+      </c>
+      <c r="C137" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="E137" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F137" s="5"/>
+      <c r="G137" s="5"/>
+      <c r="H137" s="6"/>
+      <c r="I137" s="5"/>
+    </row>
+    <row r="138" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A138" s="5"/>
+      <c r="B138" s="6" t="n">
+        <v>571</v>
+      </c>
+      <c r="C138" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="E138" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F138" s="5"/>
+      <c r="G138" s="5"/>
+      <c r="H138" s="6"/>
+      <c r="I138" s="5"/>
+    </row>
+    <row r="139" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A139" s="5"/>
+      <c r="B139" s="6" t="n">
+        <v>572</v>
+      </c>
+      <c r="C139" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E139" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F139" s="5"/>
+      <c r="G139" s="5"/>
+      <c r="H139" s="6"/>
+      <c r="I139" s="5"/>
+    </row>
+    <row r="140" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A140" s="5"/>
+      <c r="B140" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="C140" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="E140" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F140" s="5"/>
+      <c r="G140" s="5"/>
+      <c r="H140" s="6"/>
+      <c r="I140" s="5"/>
+    </row>
+    <row r="141" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A141" s="5"/>
+      <c r="B141" s="6" t="n">
+        <v>574</v>
+      </c>
+      <c r="C141" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E141" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="F141" s="5"/>
+      <c r="G141" s="5"/>
+      <c r="H141" s="6"/>
+      <c r="I141" s="5"/>
+    </row>
+    <row r="142" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A142" s="5"/>
+      <c r="B142" s="6" t="n">
+        <v>575</v>
+      </c>
+      <c r="C142" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="E142" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="F142" s="5"/>
+      <c r="G142" s="5"/>
+      <c r="H142" s="6"/>
+      <c r="I142" s="5"/>
+    </row>
+    <row r="143" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A143" s="5"/>
+      <c r="B143" s="6" t="n">
+        <v>576</v>
+      </c>
+      <c r="C143" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E143" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F143" s="5"/>
+      <c r="G143" s="5"/>
+      <c r="H143" s="6"/>
+      <c r="I143" s="5"/>
+    </row>
+    <row r="144" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A144" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B144" s="6" t="n">
+        <f aca="false">B143+C143</f>
+        <v>672</v>
+      </c>
+      <c r="C144" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E144" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="F144" s="5"/>
+      <c r="G144" s="5"/>
+      <c r="H144" s="6"/>
+      <c r="I144" s="5"/>
+    </row>
+    <row r="145" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A145" s="5"/>
+      <c r="B145" s="6" t="n">
+        <f aca="false">B144+C144</f>
+        <v>680</v>
+      </c>
+      <c r="C145" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D145" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E145" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F145" s="5"/>
+      <c r="G145" s="5"/>
+      <c r="H145" s="6"/>
+      <c r="I145" s="5"/>
+    </row>
+    <row r="146" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A146" s="5"/>
+      <c r="B146" s="6" t="n">
+        <f aca="false">B145+C145</f>
+        <v>682</v>
+      </c>
+      <c r="C146" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D146" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E146" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F146" s="5"/>
+      <c r="G146" s="5"/>
+      <c r="H146" s="6"/>
+      <c r="I146" s="5"/>
+    </row>
+    <row r="147" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A147" s="5"/>
+      <c r="B147" s="6" t="n">
+        <f aca="false">B146+C146</f>
+        <v>684</v>
+      </c>
+      <c r="C147" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E147" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="F147" s="5"/>
+      <c r="G147" s="5"/>
+      <c r="H147" s="6"/>
+      <c r="I147" s="5"/>
+    </row>
+    <row r="148" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A148" s="5"/>
+      <c r="B148" s="6" t="n">
+        <f aca="false">B147+C147</f>
+        <v>688</v>
+      </c>
+      <c r="C148" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D148" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E148" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="F148" s="5"/>
+      <c r="G148" s="5"/>
+      <c r="H148" s="6"/>
+      <c r="I148" s="5"/>
+    </row>
+    <row r="149" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A149" s="5"/>
+      <c r="B149" s="6" t="n">
+        <f aca="false">B148+C148</f>
+        <v>690</v>
+      </c>
+      <c r="C149" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D149" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E149" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F149" s="5"/>
+      <c r="G149" s="5"/>
+      <c r="H149" s="6"/>
+      <c r="I149" s="5"/>
+    </row>
+    <row r="150" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A150" s="5"/>
+      <c r="B150" s="6" t="n">
+        <f aca="false">B149+C149</f>
+        <v>692</v>
+      </c>
+      <c r="C150" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D150" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E150" s="6"/>
+      <c r="F150" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="G150" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="H150" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="I150" s="5"/>
+    </row>
+    <row r="151" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A151" s="5"/>
+      <c r="B151" s="6" t="n">
+        <f aca="false">B150+C150</f>
+        <v>704</v>
+      </c>
+      <c r="C151" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D151" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E151" s="6"/>
+      <c r="F151" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="G151" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="H151" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I151" s="5"/>
+    </row>
+    <row r="152" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A152" s="5"/>
+      <c r="B152" s="6" t="n">
+        <f aca="false">B151+C151</f>
+        <v>716</v>
+      </c>
+      <c r="C152" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D152" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E152" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="F152" s="5"/>
+      <c r="G152" s="5"/>
+      <c r="H152" s="6"/>
+      <c r="I152" s="5"/>
+    </row>
+    <row r="153" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A153" s="5"/>
+      <c r="B153" s="6" t="n">
+        <f aca="false">B152+C152</f>
+        <v>718</v>
+      </c>
+      <c r="C153" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E153" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F153" s="5"/>
+      <c r="G153" s="5"/>
+      <c r="H153" s="6"/>
+      <c r="I153" s="5"/>
+    </row>
+    <row r="154" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A154" s="5"/>
+      <c r="B154" s="6" t="n">
+        <f aca="false">B153+C153</f>
+        <v>720</v>
+      </c>
+      <c r="C154" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D154" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E154" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="F154" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="G154" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="H154" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I154" s="5"/>
+    </row>
+    <row r="155" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A155" s="5"/>
+      <c r="B155" s="6" t="n">
+        <f aca="false">B154+C154</f>
         <v>732</v>
       </c>
-      <c r="C133" s="6" t="n">
+      <c r="C155" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D133" s="5"/>
-      <c r="E133" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="F133" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="G133" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H133" s="6" t="n">
+      <c r="D155" s="5"/>
+      <c r="E155" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="F155" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="G155" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="H155" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="I133" s="5"/>
-    </row>
+      <c r="I155" s="5"/>
+    </row>
+    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
[CI] [80147]  <wifi> <feat> [RF] add SRRC policy with RF Power Calibration
</commit_message>
<xml_diff>
--- a/middleware/soc/bk7239n/sys_persist_config.xlsx
+++ b/middleware/soc/bk7239n/sys_persist_config.xlsx
@@ -321,7 +321,7 @@
     <t xml:space="preserve">0x3937E59F</t>
   </si>
   <si>
-    <t xml:space="preserve">0xCE31E2FB</t>
+    <t xml:space="preserve">0x9E7F96F4</t>
   </si>
   <si>
     <t xml:space="preserve">0xF7ECFFFF</t>
@@ -333,7 +333,7 @@
     <t xml:space="preserve">0x2F6F09E2</t>
   </si>
   <si>
-    <t xml:space="preserve">0x9E14E37F</t>
+    <t xml:space="preserve">0x9E7F4DF8</t>
   </si>
   <si>
     <t xml:space="preserve">0x44444444</t>

</xml_diff>